<commit_message>
fix: Implement flexible song name matching for Musosoup/SubmitHub data ingestion and dropdown aggregation
</commit_message>
<xml_diff>
--- a/data-backend/TSAB Metadata.xlsx
+++ b/data-backend/TSAB Metadata.xlsx
@@ -3,17 +3,18 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Cyanite Outputs" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="SubmitHub Outputs - Marbles" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">Sheet1!$A$1:$I$15</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'Cyanite Outputs'!$A$1:$I$15</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="56">
   <si>
     <t>Song</t>
   </si>
@@ -160,6 +161,27 @@
   </si>
   <si>
     <t>contemporary</t>
+  </si>
+  <si>
+    <t>Genre Composition</t>
+  </si>
+  <si>
+    <t>Percentage</t>
+  </si>
+  <si>
+    <t>Blues</t>
+  </si>
+  <si>
+    <t>Blues Rock</t>
+  </si>
+  <si>
+    <t>Southern Rock / Red Dirt</t>
+  </si>
+  <si>
+    <t>Progressive Rock</t>
+  </si>
+  <si>
+    <t>Nu Jazz / Jazztronica</t>
   </si>
 </sst>
 </file>
@@ -197,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -233,6 +255,12 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -294,7 +322,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle count="4" pivot="0" name="Sheet1-style">
+    <tableStyle count="4" pivot="0" name="Cyanite Outputs-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -308,19 +336,17 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I15" displayName="Table1" name="Table1" id="1">
-  <autoFilter ref="$A$1:$I$15">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="Marbles"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="$A$1:$I$15"/>
   <tableColumns count="9">
     <tableColumn name="Song" id="1"/>
     <tableColumn name="Main Genres" id="2"/>
@@ -332,7 +358,7 @@
     <tableColumn name="Auto-Description" id="8"/>
     <tableColumn name="Musical Era" id="9"/>
   </tableColumns>
-  <tableStyleInfo name="Sheet1-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Cyanite Outputs-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -572,7 +598,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="22.5" hidden="1" customHeight="1">
+    <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>9</v>
       </c>
@@ -601,7 +627,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" ht="22.5" hidden="1" customHeight="1">
+    <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>18</v>
       </c>
@@ -630,7 +656,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" ht="22.5" hidden="1" customHeight="1">
+    <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>27</v>
       </c>
@@ -688,7 +714,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="6" ht="22.5" hidden="1" customHeight="1">
+    <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>40</v>
       </c>
@@ -717,7 +743,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" ht="22.5" hidden="1" customHeight="1">
+    <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="9"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
@@ -727,7 +753,7 @@
       <c r="G7" s="10"/>
       <c r="H7" s="11"/>
     </row>
-    <row r="8" ht="22.5" hidden="1" customHeight="1">
+    <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="9"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
@@ -737,7 +763,7 @@
       <c r="G8" s="10"/>
       <c r="H8" s="11"/>
     </row>
-    <row r="9" ht="22.5" hidden="1" customHeight="1">
+    <row r="9" ht="22.5" customHeight="1">
       <c r="A9" s="9"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
@@ -747,7 +773,7 @@
       <c r="G9" s="10"/>
       <c r="H9" s="11"/>
     </row>
-    <row r="10" ht="22.5" hidden="1" customHeight="1">
+    <row r="10" ht="22.5" customHeight="1">
       <c r="A10" s="9"/>
       <c r="B10" s="10"/>
       <c r="C10" s="10"/>
@@ -757,7 +783,7 @@
       <c r="G10" s="10"/>
       <c r="H10" s="11"/>
     </row>
-    <row r="11" ht="22.5" hidden="1" customHeight="1">
+    <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="9"/>
       <c r="B11" s="10"/>
       <c r="C11" s="10"/>
@@ -767,7 +793,7 @@
       <c r="G11" s="10"/>
       <c r="H11" s="11"/>
     </row>
-    <row r="12" ht="22.5" hidden="1" customHeight="1">
+    <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="9"/>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
@@ -777,7 +803,7 @@
       <c r="G12" s="10"/>
       <c r="H12" s="11"/>
     </row>
-    <row r="13" ht="22.5" hidden="1" customHeight="1">
+    <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="9"/>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
@@ -787,7 +813,7 @@
       <c r="G13" s="10"/>
       <c r="H13" s="11"/>
     </row>
-    <row r="14" ht="22.5" hidden="1" customHeight="1">
+    <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="9"/>
       <c r="B14" s="10"/>
       <c r="C14" s="10"/>
@@ -797,7 +823,7 @@
       <c r="G14" s="10"/>
       <c r="H14" s="11"/>
     </row>
-    <row r="15" ht="22.5" hidden="1" customHeight="1">
+    <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="9"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -833,4 +859,67 @@
     <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="24.38"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B2" s="13">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" s="13">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="13">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="13">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="B6" s="13">
+        <v>0.08</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>